<commit_message>
Correction of some parameters in configuration files
- Some parameter values corrected in multiple configuration files.
- However, only one scenario file (75) has a change (n_icu_samples_per_week = 500->1000) which impacts the ICU 26 sites median TD results (~41.4 days -> ~39.5 days).
- The other changes are for parameter values that are not used in those scenarios, i.e. a change to the GP sampling parameters in a scenario which is only used for computing HARISS TDs.
</commit_message>
<xml_diff>
--- a/config/2026_02_18/config file record.xlsx
+++ b/config/2026_02_18/config file record.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://imperiallondon-my.sharepoint.com/personal/kdrake_ic_ac_uk/Documents/Documents/GitHub/NBPMscape/config/HARISS/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kdrake\Documents\GitHub\NBPMscape\config\2026_02_18\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="5" documentId="13_ncr:1_{C7AF26DC-B0E2-4B0D-BD3A-7ED0978896F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C729085B-7D9A-4380-A739-D4433CD82F5E}"/>
   <bookViews>
-    <workbookView xWindow="-10890" yWindow="-16095" windowWidth="25440" windowHeight="15270" xr2:uid="{4E10D132-2E59-4EE7-87E4-51CF180C7756}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{4E10D132-2E59-4EE7-87E4-51CF180C7756}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>